<commit_message>
resolved issue with vercel
</commit_message>
<xml_diff>
--- a/lista invitados.xlsx
+++ b/lista invitados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgonzalez\Downloads\b_v65DkOLGELF-1772367003108\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FCDC7A-75AA-49AF-80CD-F97ED7CCDF0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFF538C-AD85-409F-B440-DF76C2333196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44C5FF0A-3C38-4CA2-8BE7-78305C9CEF1F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$129</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="137">
   <si>
     <t>Rigoberto Espinel &amp; Señora</t>
   </si>
@@ -299,9 +299,6 @@
     <t>Sildana Rico</t>
   </si>
   <si>
-    <t xml:space="preserve">Ortensia </t>
-  </si>
-  <si>
     <t>Stella Lopez e Hija</t>
   </si>
   <si>
@@ -438,6 +435,21 @@
   </si>
   <si>
     <t>Invitados</t>
+  </si>
+  <si>
+    <t>Ortensia Gomez</t>
+  </si>
+  <si>
+    <t>Steven Perdomo &amp; Señora</t>
+  </si>
+  <si>
+    <t>Stivens Castañeda, Señora e hija</t>
+  </si>
+  <si>
+    <t>Yeimy</t>
+  </si>
+  <si>
+    <t>Edward Camilo Romero</t>
   </si>
 </sst>
 </file>
@@ -852,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99583774-8AA0-49D1-8F72-7C7187A35315}">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
@@ -861,7 +873,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>10</v>
@@ -916,472 +928,472 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>133</v>
       </c>
       <c r="B6" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="5">
         <v>3</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>85</v>
+        <v>136</v>
       </c>
       <c r="B10" s="5">
         <v>1</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B11" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B12" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B13" s="5">
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="B14" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B15" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B16" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B17" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B18" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B19" s="5">
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B20" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B21" s="5">
         <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B22" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B23" s="5">
         <v>2</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B25" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B26" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B27" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B28" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B29" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B30" s="5">
         <v>1</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B31" s="5">
         <v>1</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B32" s="5">
         <v>2</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B33" s="5">
         <v>1</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="B34" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B35" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="B36" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="B37" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="B38" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="B39" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B40" s="5">
         <v>0</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B41" s="5">
         <v>0</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B42" s="5">
         <v>0</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B43" s="5">
         <v>0</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="B44" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="B45" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>73</v>
+        <v>128</v>
       </c>
       <c r="B46" s="5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>74</v>
+        <v>129</v>
       </c>
       <c r="B47" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B48" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>80</v>
@@ -1389,10 +1401,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B49" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>80</v>
@@ -1400,10 +1412,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B50" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>80</v>
@@ -1411,10 +1423,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B51" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>80</v>
@@ -1422,64 +1434,64 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B52" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B53" s="4">
-        <v>2</v>
+      <c r="A53" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B53" s="5">
+        <v>4</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B54" s="4">
-        <v>3</v>
+      <c r="A54" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B54" s="5">
+        <v>4</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="B55" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="B56" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B57" s="5">
+      <c r="A57" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B57" s="4">
         <v>2</v>
       </c>
       <c r="C57" s="5" t="s">
@@ -1487,63 +1499,63 @@
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B58" s="5">
-        <v>1</v>
+      <c r="A58" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B58" s="4">
+        <v>3</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="3" t="s">
-        <v>1</v>
+      <c r="A59" s="5" t="s">
+        <v>2</v>
       </c>
       <c r="B59" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="3" t="s">
-        <v>112</v>
+      <c r="A60" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B60" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="3" t="s">
-        <v>113</v>
+      <c r="A61" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B61" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="3" t="s">
-        <v>114</v>
+      <c r="A62" s="5" t="s">
+        <v>5</v>
       </c>
       <c r="B62" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
-        <v>115</v>
+      <c r="A63" s="3" t="s">
+        <v>1</v>
       </c>
       <c r="B63" s="5">
         <v>0</v>
@@ -1553,8 +1565,8 @@
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
-        <v>116</v>
+      <c r="A64" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="B64" s="5">
         <v>0</v>
@@ -1564,8 +1576,8 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="5" t="s">
-        <v>117</v>
+      <c r="A65" s="3" t="s">
+        <v>112</v>
       </c>
       <c r="B65" s="5">
         <v>0</v>
@@ -1575,8 +1587,8 @@
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
-        <v>118</v>
+      <c r="A66" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="B66" s="5">
         <v>0</v>
@@ -1587,7 +1599,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B67" s="5">
         <v>0</v>
@@ -1598,7 +1610,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B68" s="5">
         <v>0</v>
@@ -1609,7 +1621,7 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B69" s="5">
         <v>0</v>
@@ -1620,54 +1632,54 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="B70" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>70</v>
+        <v>13</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>15</v>
+        <v>118</v>
       </c>
       <c r="B71" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>70</v>
+        <v>13</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>16</v>
+        <v>119</v>
       </c>
       <c r="B72" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>70</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>17</v>
+        <v>120</v>
       </c>
       <c r="B73" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>70</v>
+        <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B74" s="6">
-        <v>2</v>
+      <c r="A74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B74" s="5">
+        <v>3</v>
       </c>
       <c r="C74" s="5" t="s">
         <v>70</v>
@@ -1675,7 +1687,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B75" s="5">
         <v>2</v>
@@ -1686,7 +1698,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B76" s="5">
         <v>1</v>
@@ -1697,21 +1709,21 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B77" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C77" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B78" s="5">
-        <v>3</v>
+      <c r="A78" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B78" s="6">
+        <v>2</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>70</v>
@@ -1719,10 +1731,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B79" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>70</v>
@@ -1730,7 +1742,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B80" s="5">
         <v>1</v>
@@ -1741,7 +1753,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B81" s="5">
         <v>3</v>
@@ -1752,10 +1764,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B82" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>70</v>
@@ -1763,10 +1775,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B83" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C83" s="5" t="s">
         <v>70</v>
@@ -1774,10 +1786,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B84" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C84" s="5" t="s">
         <v>70</v>
@@ -1785,10 +1797,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B85" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C85" s="5" t="s">
         <v>70</v>
@@ -1796,21 +1808,21 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B86" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C86" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B87" s="6">
-        <v>2</v>
+      <c r="A87" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B87" s="5">
+        <v>1</v>
       </c>
       <c r="C87" s="5" t="s">
         <v>70</v>
@@ -1818,10 +1830,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B88" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C88" s="5" t="s">
         <v>70</v>
@@ -1829,20 +1841,20 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B89" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C89" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A90" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B90" s="6">
+      <c r="A90" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B90" s="5">
         <v>4</v>
       </c>
       <c r="C90" s="5" t="s">
@@ -1850,21 +1862,21 @@
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B91" s="5">
-        <v>3</v>
+      <c r="A91" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B91" s="6">
+        <v>2</v>
       </c>
       <c r="C91" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A92" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B92" s="6">
+      <c r="A92" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B92" s="5">
         <v>2</v>
       </c>
       <c r="C92" s="5" t="s">
@@ -1873,10 +1885,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B93" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C93" s="5" t="s">
         <v>70</v>
@@ -1884,10 +1896,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B94" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C94" s="5" t="s">
         <v>70</v>
@@ -1895,7 +1907,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B95" s="5">
         <v>3</v>
@@ -1905,11 +1917,11 @@
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B96" s="5">
-        <v>3</v>
+      <c r="A96" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B96" s="6">
+        <v>2</v>
       </c>
       <c r="C96" s="5" t="s">
         <v>70</v>
@@ -1917,20 +1929,20 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B97" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C97" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B98" s="5">
+      <c r="A98" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B98" s="6">
         <v>2</v>
       </c>
       <c r="C98" s="5" t="s">
@@ -1938,10 +1950,10 @@
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A99" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B99" s="6">
+      <c r="A99" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B99" s="5">
         <v>3</v>
       </c>
       <c r="C99" s="5" t="s">
@@ -1950,10 +1962,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B100" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C100" s="5" t="s">
         <v>70</v>
@@ -1961,20 +1973,20 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B101" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C101" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A102" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B102" s="6">
+      <c r="A102" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B102" s="5">
         <v>2</v>
       </c>
       <c r="C102" s="5" t="s">
@@ -1982,11 +1994,11 @@
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A103" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B103" s="5">
-        <v>4</v>
+      <c r="A103" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B103" s="6">
+        <v>3</v>
       </c>
       <c r="C103" s="5" t="s">
         <v>70</v>
@@ -1994,10 +2006,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B104" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>70</v>
@@ -2005,20 +2017,20 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B105" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C105" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A106" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B106" s="5">
+      <c r="A106" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B106" s="6">
         <v>2</v>
       </c>
       <c r="C106" s="5" t="s">
@@ -2027,20 +2039,20 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B107" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C107" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A108" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B108" s="6">
+      <c r="A108" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B108" s="5">
         <v>3</v>
       </c>
       <c r="C108" s="5" t="s">
@@ -2048,11 +2060,11 @@
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A109" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B109" s="6">
-        <v>2</v>
+      <c r="A109" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B109" s="5">
+        <v>4</v>
       </c>
       <c r="C109" s="5" t="s">
         <v>70</v>
@@ -2060,10 +2072,10 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B110" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>70</v>
@@ -2071,7 +2083,7 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B111" s="5">
         <v>2</v>
@@ -2081,22 +2093,22 @@
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A112" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B112" s="5">
-        <v>2</v>
+      <c r="A112" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B112" s="6">
+        <v>3</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A113" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B113" s="5">
-        <v>4</v>
+      <c r="A113" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B113" s="6">
+        <v>2</v>
       </c>
       <c r="C113" s="5" t="s">
         <v>70</v>
@@ -2104,10 +2116,10 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B114" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C114" s="5" t="s">
         <v>70</v>
@@ -2115,10 +2127,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B115" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>70</v>
@@ -2126,7 +2138,7 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B116" s="5">
         <v>2</v>
@@ -2137,10 +2149,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B117" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C117" s="5" t="s">
         <v>70</v>
@@ -2148,10 +2160,10 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B118" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C118" s="5" t="s">
         <v>70</v>
@@ -2159,10 +2171,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B119" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C119" s="5" t="s">
         <v>70</v>
@@ -2170,7 +2182,7 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B120" s="5">
         <v>2</v>
@@ -2181,10 +2193,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B121" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C121" s="5" t="s">
         <v>70</v>
@@ -2192,10 +2204,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B122" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C122" s="5" t="s">
         <v>70</v>
@@ -2203,10 +2215,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B123" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C123" s="5" t="s">
         <v>70</v>
@@ -2214,10 +2226,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B124" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C124" s="5" t="s">
         <v>70</v>
@@ -2225,19 +2237,63 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B125" s="5">
+        <v>2</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B126" s="5">
+        <v>2</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B127" s="5">
+        <v>3</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B128" s="5">
+        <v>5</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A129" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B125" s="5">
-        <v>2</v>
-      </c>
-      <c r="C125" s="5" t="s">
+      <c r="B129" s="5">
+        <v>2</v>
+      </c>
+      <c r="C129" s="5" t="s">
         <v>70</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C125" xr:uid="{99583774-8AA0-49D1-8F72-7C7187A35315}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C125">
-      <sortCondition ref="C1:C125"/>
+  <autoFilter ref="A1:C129" xr:uid="{99583774-8AA0-49D1-8F72-7C7187A35315}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C129">
+      <sortCondition ref="C1:C129"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>